<commit_message>
Publication figures: fix overlapping and truncated labels
- Figure 3: Table 2 compounds circled and numbered, numbers in a side column with leader lines; FDR line in legend
- Figure 4: full compound names wrapped instead of truncated; more space between panels
- Figure 6: full marker names, row height adapts to wrapped labels
- Figure S3: sample labels placed with adjustText
- Figure S4: fix x-limit (operator precedence), q values in a column outside the axes
- Table 2: No. column, numeric q sort; annotations no longer truncated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDn5T1yz4TRFaKpaKqad5Y
</commit_message>
<xml_diff>
--- a/results/publication/Tables_main.xlsx
+++ b/results/publication/Tables_main.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="89">
   <si>
     <t>Group</t>
   </si>
@@ -126,6 +126,9 @@
     <t>8.2e-05</t>
   </si>
   <si>
+    <t>No.</t>
+  </si>
+  <si>
     <t>Compound (annotation)</t>
   </si>
   <si>
@@ -165,13 +168,16 @@
     <t>Detected, % Control/BC/PC</t>
   </si>
   <si>
+    <t>C19H28O3 oxo-androstane (putatively 11-oxoetiocholanolone)</t>
+  </si>
+  <si>
     <t>unknown</t>
   </si>
   <si>
     <t>Dodecanoylcarnitine</t>
   </si>
   <si>
-    <t>Ethyl 2-amino-5-methyl-3-thiophene</t>
+    <t>Ethyl 2-amino-5-methyl-3-thiophenecarboxylate</t>
   </si>
   <si>
     <t>Biliverdin</t>
@@ -183,7 +189,7 @@
     <t>Valyl-Leucine</t>
   </si>
   <si>
-    <t>C19H28O3 oxo-androstane (putatively 11-oxoetiocholanolone)</t>
+    <t>5.beta.-Androstan-3.alpha.-ol-11,17-dione</t>
   </si>
   <si>
     <t>NCGC00380230-01_C26H40O9_2,4a,6-Trihydroxy-8-isopropyl-1,1-dimethyl-2,3,4,4a,5,10,11,11a-octahydro-1H-dibenzo[a,d][7]annulen-7-yl beta-D-glucopyranoside</t>
@@ -192,9 +198,6 @@
     <t>LAUROYLCARNITINE</t>
   </si>
   <si>
-    <t>Ethyl 2-amino-5-methyl-3-thiophenecarboxylate</t>
-  </si>
-  <si>
     <t>Unknown</t>
   </si>
   <si>
@@ -207,12 +210,12 @@
     <t>Val-Leu</t>
   </si>
   <si>
-    <t>5.beta.-Androstan-3.alpha.-ol-11,17-dione</t>
-  </si>
-  <si>
     <t>yes</t>
   </si>
   <si>
+    <t>6.3e-03</t>
+  </si>
+  <si>
     <t>1.9e-02</t>
   </si>
   <si>
@@ -234,7 +237,7 @@
     <t>4.8e-02</t>
   </si>
   <si>
-    <t>6.3e-03</t>
+    <t>0.000</t>
   </si>
   <si>
     <t>0.011</t>
@@ -256,9 +259,6 @@
   </si>
   <si>
     <t>0.004</t>
-  </si>
-  <si>
-    <t>0.000</t>
   </si>
   <si>
     <t>0.025</t>
@@ -786,10 +786,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>36</v>
       </c>
@@ -829,333 +829,360 @@
       <c r="M1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" t="s">
+      <c r="N1" t="s">
         <v>49</v>
       </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2">
+        <v>1</v>
+      </c>
       <c r="B2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2">
+        <v>287.2007</v>
+      </c>
+      <c r="E2">
+        <v>11.06</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="G2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H2">
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <v>1.25</v>
+      </c>
+      <c r="J2" t="s">
+        <v>65</v>
+      </c>
+      <c r="K2">
+        <v>0.8</v>
+      </c>
+      <c r="L2" t="s">
+        <v>73</v>
+      </c>
+      <c r="M2" t="s">
+        <v>73</v>
+      </c>
+      <c r="N2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3">
+        <v>541.2642</v>
+      </c>
+      <c r="E3">
+        <v>11.06</v>
+      </c>
+      <c r="F3">
+        <v>7</v>
+      </c>
+      <c r="G3" t="s">
+        <v>64</v>
+      </c>
+      <c r="H3">
+        <v>3</v>
+      </c>
+      <c r="I3">
+        <v>1.14</v>
+      </c>
+      <c r="J3" t="s">
+        <v>66</v>
+      </c>
+      <c r="K3">
+        <v>0.71</v>
+      </c>
+      <c r="L3" t="s">
+        <v>74</v>
+      </c>
+      <c r="M3" t="s">
+        <v>81</v>
+      </c>
+      <c r="N3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D4">
+        <v>344.2797</v>
+      </c>
+      <c r="E4">
+        <v>14.37</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>64</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="I4">
+        <v>0.93</v>
+      </c>
+      <c r="J4" t="s">
+        <v>67</v>
+      </c>
+      <c r="K4">
+        <v>0.73</v>
+      </c>
+      <c r="L4" t="s">
+        <v>75</v>
+      </c>
+      <c r="M4" t="s">
+        <v>80</v>
+      </c>
+      <c r="N4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5">
+        <v>158.027</v>
+      </c>
+      <c r="E5">
+        <v>1.42</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>64</v>
+      </c>
+      <c r="H5">
+        <v>3</v>
+      </c>
+      <c r="I5">
+        <v>-1.19</v>
+      </c>
+      <c r="J5" t="s">
+        <v>68</v>
+      </c>
+      <c r="K5">
+        <v>0.28</v>
+      </c>
+      <c r="L5" t="s">
+        <v>76</v>
+      </c>
+      <c r="M5" t="s">
+        <v>82</v>
+      </c>
+      <c r="N5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6">
+        <v>558.2914</v>
+      </c>
+      <c r="E6">
+        <v>10.76</v>
+      </c>
+      <c r="F6">
+        <v>9</v>
+      </c>
+      <c r="G6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>0.87</v>
+      </c>
+      <c r="J6" t="s">
+        <v>69</v>
+      </c>
+      <c r="K6">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="L6" t="s">
+        <v>77</v>
+      </c>
+      <c r="M6" t="s">
+        <v>83</v>
+      </c>
+      <c r="N6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7">
+        <v>583.2553</v>
+      </c>
+      <c r="E7">
+        <v>13.48</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H7">
+        <v>2</v>
+      </c>
+      <c r="I7">
+        <v>2.18</v>
+      </c>
+      <c r="J7" t="s">
+        <v>70</v>
+      </c>
+      <c r="K7">
+        <v>0.77</v>
+      </c>
+      <c r="L7" t="s">
+        <v>78</v>
+      </c>
+      <c r="M7" t="s">
+        <v>84</v>
+      </c>
+      <c r="N7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8">
+        <v>496.3397</v>
+      </c>
+      <c r="E8">
+        <v>16.71</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>64</v>
+      </c>
+      <c r="H8">
+        <v>2</v>
+      </c>
+      <c r="I8">
+        <v>1.3</v>
+      </c>
+      <c r="J8" t="s">
+        <v>71</v>
+      </c>
+      <c r="K8">
+        <v>0.79</v>
+      </c>
+      <c r="L8" t="s">
+        <v>79</v>
+      </c>
+      <c r="M8" t="s">
+        <v>73</v>
+      </c>
+      <c r="N8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
         <v>56</v>
       </c>
-      <c r="C2">
-        <v>541.2642</v>
-      </c>
-      <c r="D2">
-        <v>11.06</v>
-      </c>
-      <c r="E2">
-        <v>7</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="C9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9">
+        <v>231.1704</v>
+      </c>
+      <c r="E9">
+        <v>3.72</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" t="s">
         <v>64</v>
       </c>
-      <c r="G2">
-        <v>3</v>
-      </c>
-      <c r="H2">
-        <v>1.14</v>
-      </c>
-      <c r="I2" t="s">
-        <v>65</v>
-      </c>
-      <c r="J2">
-        <v>0.71</v>
-      </c>
-      <c r="K2" t="s">
-        <v>73</v>
-      </c>
-      <c r="L2" t="s">
-        <v>81</v>
-      </c>
-      <c r="M2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C3">
-        <v>344.2797</v>
-      </c>
-      <c r="D3">
-        <v>14.37</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G3">
+      <c r="H9">
         <v>2</v>
       </c>
-      <c r="H3">
-        <v>0.93</v>
-      </c>
-      <c r="I3" t="s">
-        <v>66</v>
-      </c>
-      <c r="J3">
-        <v>0.73</v>
-      </c>
-      <c r="K3" t="s">
-        <v>74</v>
-      </c>
-      <c r="L3" t="s">
-        <v>79</v>
-      </c>
-      <c r="M3" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C4">
-        <v>158.027</v>
-      </c>
-      <c r="D4">
-        <v>1.42</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G4">
-        <v>3</v>
-      </c>
-      <c r="H4">
-        <v>-1.19</v>
-      </c>
-      <c r="I4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J4">
-        <v>0.28</v>
-      </c>
-      <c r="K4" t="s">
-        <v>75</v>
-      </c>
-      <c r="L4" t="s">
-        <v>82</v>
-      </c>
-      <c r="M4" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C5">
-        <v>558.2914</v>
-      </c>
-      <c r="D5">
-        <v>10.76</v>
-      </c>
-      <c r="E5">
-        <v>9</v>
-      </c>
-      <c r="F5" t="s">
-        <v>64</v>
-      </c>
-      <c r="G5">
-        <v>3</v>
-      </c>
-      <c r="H5">
-        <v>0.87</v>
-      </c>
-      <c r="I5" t="s">
-        <v>68</v>
-      </c>
-      <c r="J5">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="K5" t="s">
-        <v>76</v>
-      </c>
-      <c r="L5" t="s">
-        <v>83</v>
-      </c>
-      <c r="M5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B6" t="s">
-        <v>60</v>
-      </c>
-      <c r="C6">
-        <v>583.2553</v>
-      </c>
-      <c r="D6">
-        <v>13.48</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6" t="s">
-        <v>64</v>
-      </c>
-      <c r="G6">
-        <v>2</v>
-      </c>
-      <c r="H6">
-        <v>2.18</v>
-      </c>
-      <c r="I6" t="s">
-        <v>69</v>
-      </c>
-      <c r="J6">
-        <v>0.77</v>
-      </c>
-      <c r="K6" t="s">
-        <v>77</v>
-      </c>
-      <c r="L6" t="s">
-        <v>84</v>
-      </c>
-      <c r="M6" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C7">
-        <v>496.3397</v>
-      </c>
-      <c r="D7">
-        <v>16.71</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7" t="s">
-        <v>64</v>
-      </c>
-      <c r="G7">
-        <v>2</v>
-      </c>
-      <c r="H7">
-        <v>1.3</v>
-      </c>
-      <c r="I7" t="s">
-        <v>70</v>
-      </c>
-      <c r="J7">
-        <v>0.79</v>
-      </c>
-      <c r="K7" t="s">
-        <v>78</v>
-      </c>
-      <c r="L7" t="s">
-        <v>80</v>
-      </c>
-      <c r="M7" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B8" t="s">
-        <v>62</v>
-      </c>
-      <c r="C8">
-        <v>231.1704</v>
-      </c>
-      <c r="D8">
-        <v>3.72</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8" t="s">
-        <v>64</v>
-      </c>
-      <c r="G8">
-        <v>2</v>
-      </c>
-      <c r="H8">
+      <c r="I9">
         <v>1.72</v>
       </c>
-      <c r="I8" t="s">
-        <v>71</v>
-      </c>
-      <c r="J8">
+      <c r="J9" t="s">
+        <v>72</v>
+      </c>
+      <c r="K9">
         <v>0.76</v>
-      </c>
-      <c r="K8" t="s">
-        <v>79</v>
-      </c>
-      <c r="L8" t="s">
-        <v>84</v>
-      </c>
-      <c r="M8" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B9" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9">
-        <v>287.2007</v>
-      </c>
-      <c r="D9">
-        <v>11.06</v>
-      </c>
-      <c r="E9">
-        <v>3</v>
-      </c>
-      <c r="F9" t="s">
-        <v>64</v>
-      </c>
-      <c r="G9">
-        <v>3</v>
-      </c>
-      <c r="H9">
-        <v>1.25</v>
-      </c>
-      <c r="I9" t="s">
-        <v>72</v>
-      </c>
-      <c r="J9">
-        <v>0.8</v>
-      </c>
-      <c r="K9" t="s">
-        <v>80</v>
       </c>
       <c r="L9" t="s">
         <v>80</v>
       </c>
       <c r="M9" t="s">
-        <v>85</v>
+        <v>84</v>
+      </c>
+      <c r="N9" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>